<commit_message>
Final: re-verified against final SelfCost (identical to previous), full-precision costs, dynamic text, standalone market-research deck
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PJ98fwASZjvQEuyWRiRoCu
</commit_message>
<xml_diff>
--- a/presentation/SNACKS_FINMODEL_ALL_MARGINS.xlsx
+++ b/presentation/SNACKS_FINMODEL_ALL_MARGINS.xlsx
@@ -5756,28 +5756,28 @@
         <v>42</v>
       </c>
       <c r="E4" s="93" t="n">
-        <v>1.3591</v>
+        <v>1.359143557800225</v>
       </c>
       <c r="F4" s="93" t="n">
-        <v>1.2145</v>
+        <v>1.214520885739111</v>
       </c>
       <c r="G4" s="93" t="n">
-        <v>1.3776</v>
+        <v>1.377611964085298</v>
       </c>
       <c r="H4" s="93" t="n">
-        <v>1.2554</v>
+        <v>1.255394528076464</v>
       </c>
       <c r="I4" s="93" t="n">
-        <v>61.16</v>
+        <v>61.16146010101011</v>
       </c>
       <c r="J4" s="93" t="n">
-        <v>54.65</v>
+        <v>54.65343985826001</v>
       </c>
       <c r="K4" s="93" t="n">
-        <v>61.99</v>
+        <v>61.99253838383839</v>
       </c>
       <c r="L4" s="93" t="n">
-        <v>56.49</v>
+        <v>56.49275376344086</v>
       </c>
     </row>
     <row r="5">
@@ -5800,28 +5800,28 @@
         <v>42</v>
       </c>
       <c r="E5" s="93" t="n">
-        <v>1.3591</v>
+        <v>1.359143557800225</v>
       </c>
       <c r="F5" s="93" t="n">
-        <v>1.2145</v>
+        <v>1.214520885739111</v>
       </c>
       <c r="G5" s="93" t="n">
-        <v>1.3776</v>
+        <v>1.377611964085298</v>
       </c>
       <c r="H5" s="93" t="n">
-        <v>1.2554</v>
+        <v>1.255394528076464</v>
       </c>
       <c r="I5" s="93" t="n">
-        <v>61.16</v>
+        <v>61.16146010101011</v>
       </c>
       <c r="J5" s="93" t="n">
-        <v>54.65</v>
+        <v>54.65343985826001</v>
       </c>
       <c r="K5" s="93" t="n">
-        <v>61.99</v>
+        <v>61.99253838383839</v>
       </c>
       <c r="L5" s="93" t="n">
-        <v>56.49</v>
+        <v>56.49275376344086</v>
       </c>
     </row>
     <row r="6">
@@ -5844,28 +5844,28 @@
         <v>50</v>
       </c>
       <c r="E6" s="93" t="n">
-        <v>1.0875</v>
+        <v>1.087469948082337</v>
       </c>
       <c r="F6" s="93" t="n">
-        <v>0.9443</v>
+        <v>0.9443331887794968</v>
       </c>
       <c r="G6" s="93" t="n">
-        <v>1.0665</v>
+        <v>1.066546535759898</v>
       </c>
       <c r="H6" s="93" t="n">
-        <v>0.9764</v>
+        <v>0.9763929300062772</v>
       </c>
       <c r="I6" s="93" t="n">
-        <v>48.94</v>
+        <v>48.93614766370517</v>
       </c>
       <c r="J6" s="93" t="n">
-        <v>42.49</v>
+        <v>42.49499349507735</v>
       </c>
       <c r="K6" s="93" t="n">
-        <v>47.99</v>
+        <v>47.9945941091954</v>
       </c>
       <c r="L6" s="93" t="n">
-        <v>43.94</v>
+        <v>43.93768185028247</v>
       </c>
     </row>
     <row r="7">
@@ -5888,28 +5888,28 @@
         <v>55</v>
       </c>
       <c r="E7" s="93" t="n">
-        <v>1.3593</v>
+        <v>1.359337154034587</v>
       </c>
       <c r="F7" s="93" t="n">
-        <v>1.1421</v>
+        <v>1.142106343439079</v>
       </c>
       <c r="G7" s="93" t="n">
-        <v>1.3332</v>
+        <v>1.333182678799489</v>
       </c>
       <c r="H7" s="93" t="n">
-        <v>1.2205</v>
+        <v>1.220490921217828</v>
       </c>
       <c r="I7" s="93" t="n">
-        <v>61.17</v>
+        <v>61.17017193155642</v>
       </c>
       <c r="J7" s="93" t="n">
-        <v>51.39</v>
+        <v>51.39478545475855</v>
       </c>
       <c r="K7" s="93" t="n">
-        <v>59.99</v>
+        <v>59.99322054597702</v>
       </c>
       <c r="L7" s="93" t="n">
-        <v>54.92</v>
+        <v>54.92209145480226</v>
       </c>
     </row>
     <row r="8">
@@ -5932,28 +5932,28 @@
         <v>2.5</v>
       </c>
       <c r="E8" s="93" t="n">
-        <v>0.2663</v>
+        <v>0.2662510455997877</v>
       </c>
       <c r="F8" s="93" t="n">
-        <v>0.2113</v>
+        <v>0.211296685616301</v>
       </c>
       <c r="G8" s="93" t="n">
-        <v>0.2691</v>
+        <v>0.2690826965390383</v>
       </c>
       <c r="H8" s="93" t="n">
-        <v>0.2361</v>
+        <v>0.2360541343863723</v>
       </c>
       <c r="I8" s="93" t="n">
-        <v>11.98</v>
+        <v>11.98129705199045</v>
       </c>
       <c r="J8" s="93" t="n">
-        <v>9.51</v>
+        <v>9.508350852733548</v>
       </c>
       <c r="K8" s="93" t="n">
-        <v>12.11</v>
+        <v>12.10872134425672</v>
       </c>
       <c r="L8" s="93" t="n">
-        <v>10.62</v>
+        <v>10.62243604738675</v>
       </c>
     </row>
     <row r="9">
@@ -5976,28 +5976,28 @@
         <v>2.5</v>
       </c>
       <c r="E9" s="93" t="n">
-        <v>0.2663</v>
+        <v>0.2662510455997877</v>
       </c>
       <c r="F9" s="93" t="n">
-        <v>0.2113</v>
+        <v>0.211296685616301</v>
       </c>
       <c r="G9" s="93" t="n">
-        <v>0.2691</v>
+        <v>0.2690826965390383</v>
       </c>
       <c r="H9" s="93" t="n">
-        <v>0.2361</v>
+        <v>0.2360541343863723</v>
       </c>
       <c r="I9" s="93" t="n">
-        <v>11.98</v>
+        <v>11.98129705199045</v>
       </c>
       <c r="J9" s="93" t="n">
-        <v>9.51</v>
+        <v>9.508350852733548</v>
       </c>
       <c r="K9" s="93" t="n">
-        <v>12.11</v>
+        <v>12.10872134425672</v>
       </c>
       <c r="L9" s="93" t="n">
-        <v>10.62</v>
+        <v>10.62243604738675</v>
       </c>
     </row>
     <row r="10">
@@ -6020,28 +6020,28 @@
         <v>2.5</v>
       </c>
       <c r="E10" s="93" t="n">
-        <v>0.2663</v>
+        <v>0.2662510455997877</v>
       </c>
       <c r="F10" s="93" t="n">
-        <v>0.2113</v>
+        <v>0.211296685616301</v>
       </c>
       <c r="G10" s="93" t="n">
-        <v>0.2691</v>
+        <v>0.2690826965390383</v>
       </c>
       <c r="H10" s="93" t="n">
-        <v>0.2361</v>
+        <v>0.2360541343863723</v>
       </c>
       <c r="I10" s="93" t="n">
-        <v>11.98</v>
+        <v>11.98129705199045</v>
       </c>
       <c r="J10" s="93" t="n">
-        <v>9.51</v>
+        <v>9.508350852733548</v>
       </c>
       <c r="K10" s="93" t="n">
-        <v>12.11</v>
+        <v>12.10872134425672</v>
       </c>
       <c r="L10" s="93" t="n">
-        <v>10.62</v>
+        <v>10.62243604738675</v>
       </c>
     </row>
     <row r="11">
@@ -6064,28 +6064,28 @@
         <v>5</v>
       </c>
       <c r="E11" s="93" t="n">
-        <v>0.4758</v>
+        <v>0.4757606057877072</v>
       </c>
       <c r="F11" s="93" t="n">
-        <v>0.3793</v>
+        <v>0.3792506879319993</v>
       </c>
       <c r="G11" s="93" t="n">
-        <v>0.4808</v>
+        <v>0.4808211438283309</v>
       </c>
       <c r="H11" s="93" t="n">
-        <v>0.4218</v>
+        <v>0.4218022229150905</v>
       </c>
       <c r="I11" s="93" t="n">
-        <v>21.41</v>
+        <v>21.40922726044682</v>
       </c>
       <c r="J11" s="93" t="n">
-        <v>17.07</v>
+        <v>17.06628095693997</v>
       </c>
       <c r="K11" s="93" t="n">
-        <v>21.64</v>
+        <v>21.63695147227489</v>
       </c>
       <c r="L11" s="93" t="n">
-        <v>18.98</v>
+        <v>18.98110003117907</v>
       </c>
     </row>
     <row r="12">
@@ -6108,28 +6108,28 @@
         <v>5</v>
       </c>
       <c r="E12" s="93" t="n">
-        <v>0.4758</v>
+        <v>0.4757606057877072</v>
       </c>
       <c r="F12" s="93" t="n">
-        <v>0.3793</v>
+        <v>0.3792506879319993</v>
       </c>
       <c r="G12" s="93" t="n">
-        <v>0.4808</v>
+        <v>0.4808211438283309</v>
       </c>
       <c r="H12" s="93" t="n">
-        <v>0.4218</v>
+        <v>0.4218022229150905</v>
       </c>
       <c r="I12" s="93" t="n">
-        <v>21.41</v>
+        <v>21.40922726044682</v>
       </c>
       <c r="J12" s="93" t="n">
-        <v>17.07</v>
+        <v>17.06628095693997</v>
       </c>
       <c r="K12" s="93" t="n">
-        <v>21.64</v>
+        <v>21.63695147227489</v>
       </c>
       <c r="L12" s="93" t="n">
-        <v>18.98</v>
+        <v>18.98110003117907</v>
       </c>
     </row>
     <row r="13">
@@ -6152,28 +6152,28 @@
         <v>12</v>
       </c>
       <c r="E13" s="93" t="n">
-        <v>0.9799</v>
+        <v>0.9798902628622066</v>
       </c>
       <c r="F13" s="93" t="n">
-        <v>0.7748</v>
+        <v>0.7747541457511499</v>
       </c>
       <c r="G13" s="93" t="n">
-        <v>0.9903</v>
+        <v>0.9903108371495588</v>
       </c>
       <c r="H13" s="93" t="n">
-        <v>0.8688</v>
+        <v>0.868755754365493</v>
       </c>
       <c r="I13" s="93" t="n">
-        <v>44.1</v>
+        <v>44.0950618287993</v>
       </c>
       <c r="J13" s="93" t="n">
-        <v>34.86</v>
+        <v>34.86393655880175</v>
       </c>
       <c r="K13" s="93" t="n">
-        <v>44.56</v>
+        <v>44.56398767173015</v>
       </c>
       <c r="L13" s="93" t="n">
-        <v>39.09</v>
+        <v>39.09400894644718</v>
       </c>
     </row>
     <row r="14">
@@ -6196,28 +6196,28 @@
         <v>12</v>
       </c>
       <c r="E14" s="93" t="n">
-        <v>0.9799</v>
+        <v>0.9798902628622066</v>
       </c>
       <c r="F14" s="93" t="n">
-        <v>0.7748</v>
+        <v>0.7747541457511499</v>
       </c>
       <c r="G14" s="93" t="n">
-        <v>0.9903</v>
+        <v>0.9903108371495588</v>
       </c>
       <c r="H14" s="93" t="n">
-        <v>0.8688</v>
+        <v>0.868755754365493</v>
       </c>
       <c r="I14" s="93" t="n">
-        <v>44.1</v>
+        <v>44.0950618287993</v>
       </c>
       <c r="J14" s="93" t="n">
-        <v>34.86</v>
+        <v>34.86393655880175</v>
       </c>
       <c r="K14" s="93" t="n">
-        <v>44.56</v>
+        <v>44.56398767173015</v>
       </c>
       <c r="L14" s="93" t="n">
-        <v>39.09</v>
+        <v>39.09400894644718</v>
       </c>
     </row>
     <row r="15">
@@ -6240,28 +6240,28 @@
         <v>12</v>
       </c>
       <c r="E15" s="93" t="n">
-        <v>0.9799</v>
+        <v>0.9798902628622066</v>
       </c>
       <c r="F15" s="93" t="n">
-        <v>0.7748</v>
+        <v>0.7747541457511499</v>
       </c>
       <c r="G15" s="93" t="n">
-        <v>0.9903</v>
+        <v>0.9903108371495588</v>
       </c>
       <c r="H15" s="93" t="n">
-        <v>0.8688</v>
+        <v>0.868755754365493</v>
       </c>
       <c r="I15" s="93" t="n">
-        <v>45.07</v>
+        <v>45.0749520916615</v>
       </c>
       <c r="J15" s="93" t="n">
-        <v>35.64</v>
+        <v>35.63869070455289</v>
       </c>
       <c r="K15" s="93" t="n">
-        <v>45.55</v>
+        <v>45.5542985088797</v>
       </c>
       <c r="L15" s="93" t="n">
-        <v>39.96</v>
+        <v>39.96276470081268</v>
       </c>
     </row>
     <row r="16">
@@ -6284,28 +6284,28 @@
         <v>10</v>
       </c>
       <c r="E16" s="93" t="n">
-        <v>0.9733000000000001</v>
+        <v>0.9733431683916063</v>
       </c>
       <c r="F16" s="93" t="n">
-        <v>0.7802</v>
+        <v>0.7801719811637252</v>
       </c>
       <c r="G16" s="93" t="n">
-        <v>0.9837</v>
+        <v>0.983694170707237</v>
       </c>
       <c r="H16" s="93" t="n">
-        <v>0.863</v>
+        <v>0.8629512848315115</v>
       </c>
       <c r="I16" s="93" t="n">
-        <v>43.8</v>
+        <v>43.80044257762228</v>
       </c>
       <c r="J16" s="93" t="n">
-        <v>35.11</v>
+        <v>35.10773915236764</v>
       </c>
       <c r="K16" s="93" t="n">
-        <v>44.27</v>
+        <v>44.26623768182566</v>
       </c>
       <c r="L16" s="93" t="n">
-        <v>38.83</v>
+        <v>38.83280781741801</v>
       </c>
     </row>
     <row r="17">
@@ -6328,28 +6328,28 @@
         <v>10</v>
       </c>
       <c r="E17" s="93" t="n">
-        <v>0.9733000000000001</v>
+        <v>0.9733431683916063</v>
       </c>
       <c r="F17" s="93" t="n">
-        <v>0.7802</v>
+        <v>0.7801719811637252</v>
       </c>
       <c r="G17" s="93" t="n">
-        <v>0.9837</v>
+        <v>0.983694170707237</v>
       </c>
       <c r="H17" s="93" t="n">
-        <v>0.863</v>
+        <v>0.8629512848315115</v>
       </c>
       <c r="I17" s="93" t="n">
-        <v>43.8</v>
+        <v>43.80044257762228</v>
       </c>
       <c r="J17" s="93" t="n">
-        <v>35.11</v>
+        <v>35.10773915236764</v>
       </c>
       <c r="K17" s="93" t="n">
-        <v>44.27</v>
+        <v>44.26623768182566</v>
       </c>
       <c r="L17" s="93" t="n">
-        <v>38.83</v>
+        <v>38.83280781741801</v>
       </c>
     </row>
     <row r="18">
@@ -6372,28 +6372,28 @@
         <v>30</v>
       </c>
       <c r="E18" s="93" t="n">
-        <v>0.9236</v>
+        <v>0.9235905006979264</v>
       </c>
       <c r="F18" s="93" t="n">
-        <v>0.7534</v>
+        <v>0.753392166283502</v>
       </c>
       <c r="G18" s="93" t="n">
-        <v>0.8472</v>
+        <v>0.8472482941277824</v>
       </c>
       <c r="H18" s="93" t="n">
-        <v>0.8045</v>
+        <v>0.8044771044202351</v>
       </c>
       <c r="I18" s="93" t="n">
-        <v>41.56</v>
+        <v>41.56157253140669</v>
       </c>
       <c r="J18" s="93" t="n">
-        <v>33.9</v>
+        <v>33.90264748275759</v>
       </c>
       <c r="K18" s="93" t="n">
-        <v>38.13</v>
+        <v>38.12617323575021</v>
       </c>
       <c r="L18" s="93" t="n">
-        <v>36.2</v>
+        <v>36.20146969891058</v>
       </c>
     </row>
     <row r="19">
@@ -6416,28 +6416,28 @@
         <v>30</v>
       </c>
       <c r="E19" s="93" t="n">
-        <v>0.9236</v>
+        <v>0.9235905006979264</v>
       </c>
       <c r="F19" s="93" t="n">
-        <v>0.7534</v>
+        <v>0.753392166283502</v>
       </c>
       <c r="G19" s="93" t="n">
-        <v>0.8472</v>
+        <v>0.8472482941277824</v>
       </c>
       <c r="H19" s="93" t="n">
-        <v>0.8045</v>
+        <v>0.8044771044202351</v>
       </c>
       <c r="I19" s="93" t="n">
-        <v>41.56</v>
+        <v>41.56157253140669</v>
       </c>
       <c r="J19" s="93" t="n">
-        <v>33.9</v>
+        <v>33.90264748275759</v>
       </c>
       <c r="K19" s="93" t="n">
-        <v>38.13</v>
+        <v>38.12617323575021</v>
       </c>
       <c r="L19" s="93" t="n">
-        <v>36.2</v>
+        <v>36.20146969891058</v>
       </c>
     </row>
     <row r="20">
@@ -6460,28 +6460,28 @@
         <v>30</v>
       </c>
       <c r="E20" s="93" t="n">
-        <v>0.9236</v>
+        <v>0.9235905006979264</v>
       </c>
       <c r="F20" s="93" t="n">
-        <v>0.7534</v>
+        <v>0.753392166283502</v>
       </c>
       <c r="G20" s="93" t="n">
-        <v>0.8472</v>
+        <v>0.8472482941277824</v>
       </c>
       <c r="H20" s="93" t="n">
-        <v>0.8045</v>
+        <v>0.8044771044202351</v>
       </c>
       <c r="I20" s="93" t="n">
-        <v>41.56</v>
+        <v>41.56157253140669</v>
       </c>
       <c r="J20" s="93" t="n">
-        <v>33.9</v>
+        <v>33.90264748275759</v>
       </c>
       <c r="K20" s="93" t="n">
-        <v>38.13</v>
+        <v>38.12617323575021</v>
       </c>
       <c r="L20" s="93" t="n">
-        <v>36.2</v>
+        <v>36.20146969891058</v>
       </c>
     </row>
     <row r="21">
@@ -6504,28 +6504,28 @@
         <v>50</v>
       </c>
       <c r="E21" s="93" t="n">
-        <v>1.3961</v>
+        <v>1.396119105813834</v>
       </c>
       <c r="F21" s="93" t="n">
-        <v>1.1388</v>
+        <v>1.138845974872994</v>
       </c>
       <c r="G21" s="93" t="n">
-        <v>1.2807</v>
+        <v>1.28070917633224</v>
       </c>
       <c r="H21" s="93" t="n">
-        <v>1.2161</v>
+        <v>1.216067776575522</v>
       </c>
       <c r="I21" s="93" t="n">
-        <v>62.83</v>
+        <v>62.82535976162252</v>
       </c>
       <c r="J21" s="93" t="n">
-        <v>51.25</v>
+        <v>51.24806886928473</v>
       </c>
       <c r="K21" s="93" t="n">
-        <v>57.63</v>
+        <v>57.63191293495079</v>
       </c>
       <c r="L21" s="93" t="n">
-        <v>54.72</v>
+        <v>54.72304994589847</v>
       </c>
     </row>
     <row r="22">
@@ -6548,28 +6548,28 @@
         <v>50</v>
       </c>
       <c r="E22" s="93" t="n">
-        <v>1.3961</v>
+        <v>1.396119105813834</v>
       </c>
       <c r="F22" s="93" t="n">
-        <v>1.1388</v>
+        <v>1.138845974872994</v>
       </c>
       <c r="G22" s="93" t="n">
-        <v>1.2807</v>
+        <v>1.28070917633224</v>
       </c>
       <c r="H22" s="93" t="n">
-        <v>1.2161</v>
+        <v>1.216067776575522</v>
       </c>
       <c r="I22" s="93" t="n">
-        <v>62.83</v>
+        <v>62.82535976162252</v>
       </c>
       <c r="J22" s="93" t="n">
-        <v>51.25</v>
+        <v>51.24806886928473</v>
       </c>
       <c r="K22" s="93" t="n">
-        <v>57.63</v>
+        <v>57.63191293495079</v>
       </c>
       <c r="L22" s="93" t="n">
-        <v>54.72</v>
+        <v>54.72304994589847</v>
       </c>
     </row>
     <row r="23">
@@ -6592,28 +6592,28 @@
         <v>50</v>
       </c>
       <c r="E23" s="93" t="n">
-        <v>1.3961</v>
+        <v>1.396119105813834</v>
       </c>
       <c r="F23" s="93" t="n">
-        <v>1.1388</v>
+        <v>1.138845974872994</v>
       </c>
       <c r="G23" s="93" t="n">
-        <v>1.2807</v>
+        <v>1.28070917633224</v>
       </c>
       <c r="H23" s="93" t="n">
-        <v>1.2161</v>
+        <v>1.216067776575522</v>
       </c>
       <c r="I23" s="93" t="n">
-        <v>62.83</v>
+        <v>62.82535976162252</v>
       </c>
       <c r="J23" s="93" t="n">
-        <v>51.25</v>
+        <v>51.24806886928473</v>
       </c>
       <c r="K23" s="93" t="n">
-        <v>57.63</v>
+        <v>57.63191293495079</v>
       </c>
       <c r="L23" s="93" t="n">
-        <v>54.72</v>
+        <v>54.72304994589847</v>
       </c>
     </row>
     <row r="24">
@@ -6636,28 +6636,28 @@
         <v>25</v>
       </c>
       <c r="E24" s="93" t="n">
-        <v>0.6931</v>
+        <v>0.6930977357659328</v>
       </c>
       <c r="F24" s="93" t="n">
-        <v>0.5663</v>
+        <v>0.5663367532750659</v>
       </c>
       <c r="G24" s="93" t="n">
-        <v>0.6108</v>
+        <v>0.6108170182920565</v>
       </c>
       <c r="H24" s="93" t="n">
-        <v>0.6042999999999999</v>
+        <v>0.6042850848914103</v>
       </c>
       <c r="I24" s="93" t="n">
-        <v>31.19</v>
+        <v>31.18939810946697</v>
       </c>
       <c r="J24" s="93" t="n">
-        <v>25.49</v>
+        <v>25.48515389737797</v>
       </c>
       <c r="K24" s="93" t="n">
-        <v>27.49</v>
+        <v>27.48676582314254</v>
       </c>
       <c r="L24" s="93" t="n">
-        <v>27.19</v>
+        <v>27.19282882011346</v>
       </c>
     </row>
     <row r="25">
@@ -6680,28 +6680,28 @@
         <v>25</v>
       </c>
       <c r="E25" s="93" t="n">
-        <v>0.6931</v>
+        <v>0.6930977357659328</v>
       </c>
       <c r="F25" s="93" t="n">
-        <v>0.5663</v>
+        <v>0.5663367532750659</v>
       </c>
       <c r="G25" s="93" t="n">
-        <v>0.6108</v>
+        <v>0.6108170182920565</v>
       </c>
       <c r="H25" s="93" t="n">
-        <v>0.6042999999999999</v>
+        <v>0.6042850848914103</v>
       </c>
       <c r="I25" s="93" t="n">
-        <v>31.19</v>
+        <v>31.18939810946697</v>
       </c>
       <c r="J25" s="93" t="n">
-        <v>25.49</v>
+        <v>25.48515389737797</v>
       </c>
       <c r="K25" s="93" t="n">
-        <v>27.49</v>
+        <v>27.48676582314254</v>
       </c>
       <c r="L25" s="93" t="n">
-        <v>27.19</v>
+        <v>27.19282882011346</v>
       </c>
     </row>
     <row r="26">
@@ -6724,28 +6724,28 @@
         <v>35</v>
       </c>
       <c r="E26" s="93" t="n">
-        <v>0.8943</v>
+        <v>0.8943190850160779</v>
       </c>
       <c r="F26" s="93" t="n">
-        <v>0.7308</v>
+        <v>0.7307568505113264</v>
       </c>
       <c r="G26" s="93" t="n">
-        <v>0.7881</v>
+        <v>0.7881472771717466</v>
       </c>
       <c r="H26" s="93" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.7797262535444972</v>
       </c>
       <c r="I26" s="93" t="n">
-        <v>40.24</v>
+        <v>40.24435882572351</v>
       </c>
       <c r="J26" s="93" t="n">
-        <v>32.88</v>
+        <v>32.88405827300969</v>
       </c>
       <c r="K26" s="93" t="n">
-        <v>35.47</v>
+        <v>35.4666274727286</v>
       </c>
       <c r="L26" s="93" t="n">
-        <v>35.09</v>
+        <v>35.08768140950237</v>
       </c>
     </row>
     <row r="27">
@@ -6768,28 +6768,28 @@
         <v>35</v>
       </c>
       <c r="E27" s="93" t="n">
-        <v>0.8943</v>
+        <v>0.8943190850160779</v>
       </c>
       <c r="F27" s="93" t="n">
-        <v>0.7008</v>
+        <v>0.700830283294026</v>
       </c>
       <c r="G27" s="93" t="n">
-        <v>0.7881</v>
+        <v>0.7881472771717466</v>
       </c>
       <c r="H27" s="93" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.7797262535444972</v>
       </c>
       <c r="I27" s="93" t="n">
-        <v>40.24</v>
+        <v>40.24435882572351</v>
       </c>
       <c r="J27" s="93" t="n">
-        <v>31.54</v>
+        <v>31.53736274823117</v>
       </c>
       <c r="K27" s="93" t="n">
-        <v>35.47</v>
+        <v>35.4666274727286</v>
       </c>
       <c r="L27" s="93" t="n">
-        <v>35.09</v>
+        <v>35.08768140950237</v>
       </c>
     </row>
     <row r="28">
@@ -6812,28 +6812,28 @@
         <v>35</v>
       </c>
       <c r="E28" s="93" t="n">
-        <v>0.8943</v>
+        <v>0.8943190850160779</v>
       </c>
       <c r="F28" s="93" t="n">
-        <v>0.7008</v>
+        <v>0.700830283294026</v>
       </c>
       <c r="G28" s="93" t="n">
-        <v>0.7881</v>
+        <v>0.7881472771717466</v>
       </c>
       <c r="H28" s="93" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.7797262535444972</v>
       </c>
       <c r="I28" s="93" t="n">
-        <v>40.24</v>
+        <v>40.24435882572351</v>
       </c>
       <c r="J28" s="93" t="n">
-        <v>31.54</v>
+        <v>31.53736274823117</v>
       </c>
       <c r="K28" s="93" t="n">
-        <v>35.47</v>
+        <v>35.4666274727286</v>
       </c>
       <c r="L28" s="93" t="n">
-        <v>35.09</v>
+        <v>35.08768140950237</v>
       </c>
     </row>
     <row r="29">
@@ -6856,28 +6856,28 @@
         <v>70</v>
       </c>
       <c r="E29" s="93" t="n">
-        <v>1.811</v>
+        <v>1.810977907140197</v>
       </c>
       <c r="F29" s="93" t="n">
-        <v>1.4192</v>
+        <v>1.419176017483534</v>
       </c>
       <c r="G29" s="93" t="n">
-        <v>1.596</v>
+        <v>1.595968963269315</v>
       </c>
       <c r="H29" s="93" t="n">
-        <v>1.5789</v>
+        <v>1.578924490450455</v>
       </c>
       <c r="I29" s="93" t="n">
-        <v>81.48999999999999</v>
+        <v>81.49400582130886</v>
       </c>
       <c r="J29" s="93" t="n">
-        <v>63.86</v>
+        <v>63.86292078675902</v>
       </c>
       <c r="K29" s="93" t="n">
-        <v>71.81999999999999</v>
+        <v>71.81860334711915</v>
       </c>
       <c r="L29" s="93" t="n">
-        <v>71.05</v>
+        <v>71.05160207027048</v>
       </c>
     </row>
     <row r="30">
@@ -6900,28 +6900,28 @@
         <v>70</v>
       </c>
       <c r="E30" s="93" t="n">
-        <v>1.811</v>
+        <v>1.810977907140197</v>
       </c>
       <c r="F30" s="93" t="n">
-        <v>1.4192</v>
+        <v>1.419176017483534</v>
       </c>
       <c r="G30" s="93" t="n">
-        <v>1.596</v>
+        <v>1.595968963269315</v>
       </c>
       <c r="H30" s="93" t="n">
-        <v>1.5789</v>
+        <v>1.578924490450455</v>
       </c>
       <c r="I30" s="93" t="n">
-        <v>81.48999999999999</v>
+        <v>81.49400582130886</v>
       </c>
       <c r="J30" s="93" t="n">
-        <v>63.86</v>
+        <v>63.86292078675902</v>
       </c>
       <c r="K30" s="93" t="n">
-        <v>71.81999999999999</v>
+        <v>71.81860334711915</v>
       </c>
       <c r="L30" s="93" t="n">
-        <v>71.05</v>
+        <v>71.05160207027048</v>
       </c>
     </row>
     <row r="31">
@@ -6944,28 +6944,28 @@
         <v>70</v>
       </c>
       <c r="E31" s="93" t="n">
-        <v>1.811</v>
+        <v>1.810977907140197</v>
       </c>
       <c r="F31" s="93" t="n">
-        <v>1.4192</v>
+        <v>1.419176017483534</v>
       </c>
       <c r="G31" s="93" t="n">
-        <v>1.596</v>
+        <v>1.595968963269315</v>
       </c>
       <c r="H31" s="93" t="n">
-        <v>1.5789</v>
+        <v>1.578924490450455</v>
       </c>
       <c r="I31" s="93" t="n">
-        <v>81.48999999999999</v>
+        <v>81.49400582130886</v>
       </c>
       <c r="J31" s="93" t="n">
-        <v>63.86</v>
+        <v>63.86292078675902</v>
       </c>
       <c r="K31" s="93" t="n">
-        <v>71.81999999999999</v>
+        <v>71.81860334711915</v>
       </c>
       <c r="L31" s="93" t="n">
-        <v>71.05</v>
+        <v>71.05160207027048</v>
       </c>
     </row>
   </sheetData>

</xml_diff>